<commit_message>
docs(backlog): mark refund operations complete
</commit_message>
<xml_diff>
--- a/outputs/launch-hardening/Vitorize_Launch_Hardening_Backlog.xlsx
+++ b/outputs/launch-hardening/Vitorize_Launch_Hardening_Backlog.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch Hardening" sheetId="1" r:id="R689b316e174e4172"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch Hardening" sheetId="1" r:id="R72c8c685fc7a4049"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -801,15 +801,19 @@
         </x:is>
       </x:c>
       <x:c r="G10" s="3" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="H10" s="3" t="str">
-        <x:v>Refund/reconcile APIs exist; operator UI screens remain open.</x:v>
-      </x:c>
-      <x:c r="I10" s="3" t="str"/>
-      <x:c r="J10" s="3" t="str"/>
+        <x:v>Admin payment details expose refund eligibility, reason/method input, persisted refund/audit history, manual gateway completion, wallet refunds, and reconciliation. FinanceManage protects money-moving actions; server locks and idempotency prevent duplicates.</x:v>
+      </x:c>
+      <x:c r="I10" s="3" t="str">
+        <x:v>AdminPaymentsController; PaymentsController; PaymentService; AdminPaymentReadService; Admin Payments UI; finance integration tests</x:v>
+      </x:c>
+      <x:c r="J10" s="3" t="str">
+        <x:v>bc43474, 928bb81</x:v>
+      </x:c>
       <x:c r="K10" s="3" t="str">
-        <x:v>Existing finance integration tests only</x:v>
+        <x:v>Release build; unit 409/409; integration 114/114; Admin Playwright 7/7</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="44" customHeight="1">

</xml_diff>

<commit_message>
docs(backlog): mark support ticket semantics complete
</commit_message>
<xml_diff>
--- a/outputs/launch-hardening/Vitorize_Launch_Hardening_Backlog.xlsx
+++ b/outputs/launch-hardening/Vitorize_Launch_Hardening_Backlog.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch Hardening" sheetId="1" r:id="R72c8c685fc7a4049"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch Hardening" sheetId="1" r:id="R6a6cb7b52f9243d2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -942,19 +942,19 @@
         </x:is>
       </x:c>
       <x:c r="G13" s="3" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="H13" s="3" t="str">
-        <x:v>One idempotent support ticket per order exists; multi-item assignment/semantics still need product-policy confirmation.</x:v>
+        <x:v>Exactly one automatic fulfilment ticket is created per qualifying order, with every SupportRequired OrderItem linked to it. Customer-created order tickets stay separate. A filtered unique database index, payment idempotency, and safe retry preserve the invariant under replay and concurrency.</x:v>
       </x:c>
       <x:c r="I13" s="3" t="str">
-        <x:v>PaymentService; PaymentDeliveryIntegrationTests</x:v>
+        <x:v>V0007; Ticket/OrderItem model; DbContext; PaymentService; TicketService; ticket DTOs and Admin/Customer ticket UI; support integration and Playwright tests</x:v>
       </x:c>
       <x:c r="J13" s="3" t="str">
-        <x:v>39024e2</x:v>
+        <x:v>ffa9658, 058148f, 24a149f, aed83ff</x:v>
       </x:c>
       <x:c r="K13" s="3" t="str">
-        <x:v>Existing support integration coverage</x:v>
+        <x:v>Release build 0 warnings; unit 410/410; SQL integration 117/117; focused browser Customer/Admin support flow 1/1 (57.1s); clean migration + upgrade rehearsal verified</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="44" customHeight="1">

</xml_diff>

<commit_message>
docs(backlog): mark storefront filters complete
</commit_message>
<xml_diff>
--- a/outputs/launch-hardening/Vitorize_Launch_Hardening_Backlog.xlsx
+++ b/outputs/launch-hardening/Vitorize_Launch_Hardening_Backlog.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch Hardening" sheetId="1" r:id="R6a6cb7b52f9243d2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch Hardening" sheetId="1" r:id="Rcf39f464224d43cf"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -989,15 +989,19 @@
         </x:is>
       </x:c>
       <x:c r="G14" s="3" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="H14" s="3" t="str">
-        <x:v>Core filters/pagination exist but catalog refinements are still partly client-side.</x:v>
-      </x:c>
-      <x:c r="I14" s="3" t="str"/>
-      <x:c r="J14" s="3" t="str"/>
+        <x:v>Storefront paging, counts, product type, delivery, verification, price, availability, and discount-tier filters now execute in the public catalog query. Invalid price ranges and discount thresholds are rejected server-side; the UI only owns filter state.</x:v>
+      </x:c>
+      <x:c r="I14" s="3" t="str">
+        <x:v>ProductFilterDto; ProductService; ShopBrowser; catalog unit and SQL integration tests</x:v>
+      </x:c>
+      <x:c r="J14" s="3" t="str">
+        <x:v>9f885dc</x:v>
+      </x:c>
       <x:c r="K14" s="3" t="str">
-        <x:v>Audit evidence retained</x:v>
+        <x:v>Release build 0 warnings; focused unit 3/3; SQL-backed catalog API integration 1/1; storefront Playwright 1/1</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="44" customHeight="1">

</xml_diff>

<commit_message>
docs(backlog): record admin paging progress
</commit_message>
<xml_diff>
--- a/outputs/launch-hardening/Vitorize_Launch_Hardening_Backlog.xlsx
+++ b/outputs/launch-hardening/Vitorize_Launch_Hardening_Backlog.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch Hardening" sheetId="1" r:id="Rcf39f464224d43cf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch Hardening" sheetId="1" r:id="Raf5224dd7f254b3d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1167,15 +1167,19 @@
         </x:is>
       </x:c>
       <x:c r="G18" s="3" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="H18" s="3" t="str">
-        <x:v>Several admin screens still load unbounded lists or use client paging.</x:v>
-      </x:c>
-      <x:c r="I18" s="3" t="str"/>
-      <x:c r="J18" s="3" t="str"/>
+        <x:v>Completed inventory in docs/REQ-010-ADMIN-PAGING-INVENTORY.md. Products, orders, payments, wallets, tickets, verification, and audit/error/security operational logs now use SQL-side filtered, counted, stable paged endpoints; legacy endpoints remain compatible. Notifications and coupons now expose the same bounded contract. Remaining: migrate their UI/export semantics, bounded lookup sources, focused paging tests, and full verification.</x:v>
+      </x:c>
+      <x:c r="I18" s="3" t="str">
+        <x:v>Admin paging inventory; Admin Products/Orders/Payments/Wallets/Tickets/Verifications/AuditLogs/ErrorLogs/SecurityLogs; paged controllers and read services</x:v>
+      </x:c>
+      <x:c r="J18" s="3" t="str">
+        <x:v>8b5fdf7, a885f5c, 02d3354</x:v>
+      </x:c>
       <x:c r="K18" s="3" t="str">
-        <x:v>Repository inspection</x:v>
+        <x:v>Release builds passed (0 warnings after incremental); focused SQL AdminCatalog suite 3/3</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="44" customHeight="1">

</xml_diff>

<commit_message>
docs(backlog): update admin paging inventory
</commit_message>
<xml_diff>
--- a/outputs/launch-hardening/Vitorize_Launch_Hardening_Backlog.xlsx
+++ b/outputs/launch-hardening/Vitorize_Launch_Hardening_Backlog.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch Hardening" sheetId="1" r:id="Raf5224dd7f254b3d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch Hardening" sheetId="1" r:id="R6702fc8ea6514a4a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1170,16 +1170,16 @@
         <x:v>In Progress</x:v>
       </x:c>
       <x:c r="H18" s="3" t="str">
-        <x:v>Completed inventory in docs/REQ-010-ADMIN-PAGING-INVENTORY.md. Products, orders, payments, wallets, tickets, verification, and audit/error/security operational logs now use SQL-side filtered, counted, stable paged endpoints; legacy endpoints remain compatible. Notifications and coupons now expose the same bounded contract. Remaining: migrate their UI/export semantics, bounded lookup sources, focused paging tests, and full verification.</x:v>
+        <x:v>Completed inventory in docs/REQ-010-ADMIN-PAGING-INVENTORY.md. Products, orders, payments, wallets, tickets, verification, notifications, coupons, and audit/error/security operational logs now use SQL-side filtered, counted, stable paged endpoints; legacy endpoints remain compatible. Gift-code product selection uses a dedicated bounded lookup. Remaining: detail-history paging, explicit export semantics, focused paging tests, and full verification.</x:v>
       </x:c>
       <x:c r="I18" s="3" t="str">
-        <x:v>Admin paging inventory; Admin Products/Orders/Payments/Wallets/Tickets/Verifications/AuditLogs/ErrorLogs/SecurityLogs; paged controllers and read services</x:v>
+        <x:v>Admin paging inventory; Admin Products/Orders/Payments/Wallets/Tickets/Verifications/Notifications/Coupons/AuditLogs/ErrorLogs/SecurityLogs; paged controllers/read services; GiftCodes lookup</x:v>
       </x:c>
       <x:c r="J18" s="3" t="str">
-        <x:v>8b5fdf7, a885f5c, 02d3354</x:v>
+        <x:v>8b5fdf7, a885f5c, 02d3354, cd98354, eaee518</x:v>
       </x:c>
       <x:c r="K18" s="3" t="str">
-        <x:v>Release builds passed (0 warnings after incremental); focused SQL AdminCatalog suite 3/3</x:v>
+        <x:v>Release builds passed (0 warnings after incremental); focused SQL AdminCatalog suite 3/3; new SQL test host currently hangs before execution and was not retained</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="44" customHeight="1">

</xml_diff>